<commit_message>
Renumera IDs das iniciativas para 1–79 (sem lacunas)
- gen_data: após exclusões/overrides/PRE/FORA_NE/ALT_LOCAIS, renumera os IDs
  sequencialmente (1..N), eliminando as lacunas de 8/28/29
- Invalida seleção antiga no navegador (chave localStorage pte_sel2) para evitar
  mapeamento incorreto com os IDs antigos
- Regenera iniciativas.js e PTE2026_base_limpa.xlsx
- Cache-busting para v=27

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012qKixxvEYzG5RpjsaQG5UL
</commit_message>
<xml_diff>
--- a/PTE2026_base_limpa.xlsx
+++ b/PTE2026_base_limpa.xlsx
@@ -1764,7 +1764,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -2076,7 +2076,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -2231,7 +2231,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -2391,7 +2391,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -2864,7 +2864,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -3182,7 +3182,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -3334,7 +3334,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -3485,7 +3485,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -3646,7 +3646,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -3806,7 +3806,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -3963,7 +3963,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
@@ -4120,7 +4120,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -4282,7 +4282,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -4439,7 +4439,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -4602,7 +4602,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -4766,7 +4766,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -4925,7 +4925,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -5083,7 +5083,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -5245,7 +5245,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -5402,7 +5402,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -5566,7 +5566,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -5721,7 +5721,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -5877,7 +5877,7 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -6034,7 +6034,7 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
@@ -6196,7 +6196,7 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -6357,7 +6357,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
@@ -6516,7 +6516,7 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -6672,7 +6672,7 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
@@ -6829,7 +6829,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -6985,7 +6985,7 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -7144,7 +7144,7 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -7301,7 +7301,7 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
@@ -7459,7 +7459,7 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -7617,7 +7617,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
@@ -7930,7 +7930,7 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
@@ -8091,7 +8091,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
@@ -8246,7 +8246,7 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
@@ -8410,7 +8410,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
@@ -8573,7 +8573,7 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
@@ -8728,7 +8728,7 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
@@ -8883,7 +8883,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
@@ -9043,7 +9043,7 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
@@ -9202,7 +9202,7 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
@@ -9361,7 +9361,7 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
@@ -9518,7 +9518,7 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
@@ -9673,7 +9673,7 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
@@ -9828,7 +9828,7 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
@@ -9983,7 +9983,7 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
@@ -10138,7 +10138,7 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
@@ -10293,7 +10293,7 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
@@ -10452,7 +10452,7 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
@@ -10611,7 +10611,7 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
@@ -10770,7 +10770,7 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
@@ -10925,7 +10925,7 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
@@ -11080,7 +11080,7 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
@@ -11235,7 +11235,7 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
@@ -11390,7 +11390,7 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
@@ -11549,7 +11549,7 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
@@ -11704,7 +11704,7 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
@@ -11863,7 +11863,7 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
@@ -12022,7 +12022,7 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
@@ -12181,7 +12181,7 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
@@ -12336,7 +12336,7 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
@@ -12491,7 +12491,7 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
@@ -12646,7 +12646,7 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
@@ -12801,7 +12801,7 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
@@ -12956,7 +12956,7 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Remove a pré-seleção estática (as 31 da matriz) de toda a base
- gen_data: remove o dicionário PRE, os campos preselecionada/pre_ufs dos itens e
  meta.preselecionadas; a pré-seleção passa a existir só via aba Seleção
- Planilha-base limpa: remove as colunas "Pré-selecionada" e "UFs (pré-seleção)"
- iniciativas.js sem qualquer resíduo de preselecionada/pre_ufs
- Painel inalterado: "pré-selecionada" = escolha da aba Seleção (dinâmico)
- Cache-busting para v=28

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012qKixxvEYzG5RpjsaQG5UL
</commit_message>
<xml_diff>
--- a/PTE2026_base_limpa.xlsx
+++ b/PTE2026_base_limpa.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Iniciativas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Iniciativas'!$A$1:$AK$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Iniciativas'!$A$1:$AI$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK80"/>
+  <dimension ref="A1:AI80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -469,8 +469,6 @@
     <col width="12" customWidth="1" min="33" max="33"/>
     <col width="30" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="12" customWidth="1" min="36" max="36"/>
-    <col width="12" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -646,16 +644,6 @@
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>Pré-selecionada</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>UFs (pré-seleção)</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
           <t>Sede fora do NE</t>
         </is>
       </c>
@@ -807,16 +795,6 @@
       </c>
       <c r="AI2" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -970,12 +948,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
-      <c r="AK3" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1122,16 +1094,6 @@
         </is>
       </c>
       <c r="AI4" s="2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ4" s="2" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="AK4" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -1286,12 +1248,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
-      <c r="AK5" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1438,12 +1394,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
-      <c r="AK6" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1591,16 +1541,6 @@
       </c>
       <c r="AI7" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ7" s="2" t="inlineStr">
-        <is>
-          <t>RN</t>
-        </is>
-      </c>
-      <c r="AK7" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -1755,12 +1695,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
-      <c r="AK8" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1903,16 +1837,6 @@
       </c>
       <c r="AI9" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ9" s="2" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="AK9" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -2059,16 +1983,6 @@
         </is>
       </c>
       <c r="AI10" s="2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ10" s="2" t="inlineStr">
-        <is>
-          <t>CE, RN, PB, PE, AL, BA</t>
-        </is>
-      </c>
-      <c r="AK10" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -2219,12 +2133,6 @@
       </c>
       <c r="AI11" s="2" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ11" s="2" t="inlineStr"/>
-      <c r="AK11" s="2" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
@@ -2374,16 +2282,6 @@
         </is>
       </c>
       <c r="AI12" s="2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ12" s="2" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="AK12" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -2535,16 +2433,6 @@
       </c>
       <c r="AI13" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ13" s="2" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="AK13" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -2700,12 +2588,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ14" s="2" t="inlineStr"/>
-      <c r="AK14" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -2855,12 +2737,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ15" s="2" t="inlineStr"/>
-      <c r="AK15" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -3007,16 +2883,6 @@
       </c>
       <c r="AI16" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ16" s="2" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="AK16" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -3166,16 +3032,6 @@
       </c>
       <c r="AI17" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ17" s="2" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="AK17" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -3325,12 +3181,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ18" s="2" t="inlineStr"/>
-      <c r="AK18" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -3473,12 +3323,6 @@
       </c>
       <c r="AI19" s="2" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ19" s="2" t="inlineStr"/>
-      <c r="AK19" s="2" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
@@ -3630,16 +3474,6 @@
       </c>
       <c r="AI20" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ20" s="2" t="inlineStr">
-        <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="AK20" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -3790,16 +3624,6 @@
       </c>
       <c r="AI21" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ21" s="2" t="inlineStr">
-        <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="AK21" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -3954,12 +3778,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ22" s="2" t="inlineStr"/>
-      <c r="AK22" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -4111,12 +3929,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ23" s="2" t="inlineStr"/>
-      <c r="AK23" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -4266,16 +4078,6 @@
       </c>
       <c r="AI24" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ24" s="2" t="inlineStr">
-        <is>
-          <t>PB, PE</t>
-        </is>
-      </c>
-      <c r="AK24" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -4426,12 +4228,6 @@
         </is>
       </c>
       <c r="AI25" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ25" s="2" t="inlineStr"/>
-      <c r="AK25" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -4593,12 +4389,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ26" s="2" t="inlineStr"/>
-      <c r="AK26" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -4749,16 +4539,6 @@
         </is>
       </c>
       <c r="AI27" s="2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ27" s="2" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="AK27" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -4916,12 +4696,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ28" s="2" t="inlineStr"/>
-      <c r="AK28" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -5074,12 +4848,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ29" s="2" t="inlineStr"/>
-      <c r="AK29" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -5229,16 +4997,6 @@
       </c>
       <c r="AI30" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ30" s="2" t="inlineStr">
-        <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="AK30" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -5389,12 +5147,6 @@
         </is>
       </c>
       <c r="AI31" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ31" s="2" t="inlineStr"/>
-      <c r="AK31" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -5550,16 +5302,6 @@
       </c>
       <c r="AI32" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ32" s="2" t="inlineStr">
-        <is>
-          <t>RN</t>
-        </is>
-      </c>
-      <c r="AK32" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -5712,12 +5454,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ33" s="2" t="inlineStr"/>
-      <c r="AK33" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -5868,12 +5604,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ34" s="2" t="inlineStr"/>
-      <c r="AK34" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -6025,12 +5755,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ35" s="2" t="inlineStr"/>
-      <c r="AK35" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -6180,16 +5904,6 @@
       </c>
       <c r="AI36" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ36" s="2" t="inlineStr">
-        <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="AK36" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -6340,16 +6054,6 @@
         </is>
       </c>
       <c r="AI37" s="2" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ37" s="2" t="inlineStr">
-        <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="AK37" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -6507,12 +6211,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ38" s="2" t="inlineStr"/>
-      <c r="AK38" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -6663,12 +6361,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ39" s="2" t="inlineStr"/>
-      <c r="AK39" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -6820,12 +6512,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ40" s="2" t="inlineStr"/>
-      <c r="AK40" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -6972,12 +6658,6 @@
         </is>
       </c>
       <c r="AI41" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ41" s="2" t="inlineStr"/>
-      <c r="AK41" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -7135,12 +6815,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ42" s="2" t="inlineStr"/>
-      <c r="AK42" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -7292,12 +6966,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ43" s="2" t="inlineStr"/>
-      <c r="AK43" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -7450,12 +7118,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ44" s="2" t="inlineStr"/>
-      <c r="AK44" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -7601,16 +7263,6 @@
       </c>
       <c r="AI45" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ45" s="2" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="AK45" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -7764,12 +7416,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ46" s="2" t="inlineStr"/>
-      <c r="AK46" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -7917,12 +7563,6 @@
         </is>
       </c>
       <c r="AI47" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ47" s="2" t="inlineStr"/>
-      <c r="AK47" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -8075,16 +7715,6 @@
       </c>
       <c r="AI48" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ48" s="2" t="inlineStr">
-        <is>
-          <t>SE</t>
-        </is>
-      </c>
-      <c r="AK48" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -8233,12 +7863,6 @@
         </is>
       </c>
       <c r="AI49" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ49" s="2" t="inlineStr"/>
-      <c r="AK49" s="2" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
@@ -8394,16 +8018,6 @@
       </c>
       <c r="AI50" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ50" s="2" t="inlineStr">
-        <is>
-          <t>PI, CE</t>
-        </is>
-      </c>
-      <c r="AK50" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -8557,16 +8171,6 @@
       </c>
       <c r="AI51" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ51" s="2" t="inlineStr">
-        <is>
-          <t>PB</t>
-        </is>
-      </c>
-      <c r="AK51" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -8719,12 +8323,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ52" s="2" t="inlineStr"/>
-      <c r="AK52" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -8874,12 +8472,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ53" s="2" t="inlineStr"/>
-      <c r="AK53" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -9027,16 +8619,6 @@
       </c>
       <c r="AI54" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ54" s="2" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="AK54" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -9186,16 +8768,6 @@
       </c>
       <c r="AI55" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ55" s="2" t="inlineStr">
-        <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="AK55" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -9345,16 +8917,6 @@
       </c>
       <c r="AI56" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ56" s="2" t="inlineStr">
-        <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="AK56" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -9506,12 +9068,6 @@
       </c>
       <c r="AI57" s="2" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ57" s="2" t="inlineStr"/>
-      <c r="AK57" s="2" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
@@ -9661,12 +9217,6 @@
       </c>
       <c r="AI58" s="2" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ58" s="2" t="inlineStr"/>
-      <c r="AK58" s="2" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
@@ -9819,12 +9369,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ59" s="2" t="inlineStr"/>
-      <c r="AK59" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -9974,12 +9518,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ60" s="2" t="inlineStr"/>
-      <c r="AK60" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -10129,12 +9667,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ61" s="2" t="inlineStr"/>
-      <c r="AK61" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -10284,12 +9816,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ62" s="2" t="inlineStr"/>
-      <c r="AK62" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -10436,16 +9962,6 @@
       </c>
       <c r="AI63" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ63" s="2" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="AK63" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -10595,16 +10111,6 @@
       </c>
       <c r="AI64" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ64" s="2" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="AK64" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -10754,16 +10260,6 @@
       </c>
       <c r="AI65" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ65" s="2" t="inlineStr">
-        <is>
-          <t>AL</t>
-        </is>
-      </c>
-      <c r="AK65" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -10916,12 +10412,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ66" s="2" t="inlineStr"/>
-      <c r="AK66" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -11071,12 +10561,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ67" s="2" t="inlineStr"/>
-      <c r="AK67" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -11223,12 +10707,6 @@
       </c>
       <c r="AI68" s="2" t="inlineStr">
         <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AJ68" s="2" t="inlineStr"/>
-      <c r="AK68" s="2" t="inlineStr">
-        <is>
           <t>Sim</t>
         </is>
       </c>
@@ -11381,12 +10859,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ69" s="2" t="inlineStr"/>
-      <c r="AK69" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -11533,16 +11005,6 @@
       </c>
       <c r="AI70" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ70" s="2" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="AK70" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -11695,12 +11157,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ71" s="2" t="inlineStr"/>
-      <c r="AK71" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -11847,16 +11303,6 @@
       </c>
       <c r="AI72" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ72" s="2" t="inlineStr">
-        <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="AK72" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -12006,16 +11452,6 @@
       </c>
       <c r="AI73" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ73" s="2" t="inlineStr">
-        <is>
-          <t>SE</t>
-        </is>
-      </c>
-      <c r="AK73" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -12165,16 +11601,6 @@
       </c>
       <c r="AI74" s="2" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="AJ74" s="2" t="inlineStr">
-        <is>
-          <t>PB</t>
-        </is>
-      </c>
-      <c r="AK74" s="2" t="inlineStr">
-        <is>
           <t>Não</t>
         </is>
       </c>
@@ -12327,12 +11753,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ75" s="2" t="inlineStr"/>
-      <c r="AK75" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -12482,12 +11902,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ76" s="2" t="inlineStr"/>
-      <c r="AK76" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -12637,12 +12051,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ77" s="2" t="inlineStr"/>
-      <c r="AK77" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -12792,12 +12200,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ78" s="2" t="inlineStr"/>
-      <c r="AK78" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -12947,12 +12349,6 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ79" s="2" t="inlineStr"/>
-      <c r="AK79" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -13102,15 +12498,9 @@
           <t>Não</t>
         </is>
       </c>
-      <c r="AJ80" s="2" t="inlineStr"/>
-      <c r="AK80" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK1"/>
+  <autoFilter ref="A1:AI1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sertão Vivo: reclassifica para eixo 6 (NIVA) + Salvador como local secundário
- EIXO_OVERRIDES/EIXO_SEC_OVERRIDES: eixo principal = Nova Infraestrutura
  Verde-Azul e Adaptação Climática (NIVA); secundário = BIO (swap)
- ALT_LOCAIS: Rio de Janeiro (sede) + Salvador (BA) como 2º local
- Regenera iniciativas.js e a planilha-base
- Cache-busting para v=32

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012qKixxvEYzG5RpjsaQG5UL
</commit_message>
<xml_diff>
--- a/PTE2026_base_limpa.xlsx
+++ b/PTE2026_base_limpa.xlsx
@@ -2666,12 +2666,12 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Bioeconomia e Sistemas Agroalimentares Adaptados</t>
+          <t>Nova Infraestrutura Verde-Azul e Adaptação Climática</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>NIVA</t>
+          <t>BIO</t>
         </is>
       </c>
       <c r="S15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Multi-local: Captação de Água da ASA e Reecatingar (municípios do sertão BA)
- Captação de Água da ASA: Remanso, Pilão Arcado e Sento Sé (BA)
- Reecatingar: Canudos, Uauá, Curaçá, Casa Nova, Remanso, Sento Sé e Sobradinho (BA)
- Município primário das iniciativas multi-local passa a refletir o 1º local
- Regenera iniciativas.js e a planilha-base; cache v=34

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012qKixxvEYzG5RpjsaQG5UL
</commit_message>
<xml_diff>
--- a/PTE2026_base_limpa.xlsx
+++ b/PTE2026_base_limpa.xlsx
@@ -3993,7 +3993,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Remígio (PB) / Araripina (PE)</t>
+          <t>Remígio</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Salvador, Fortaleza</t>
+          <t>Salvador</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
@@ -5958,10 +5958,10 @@
         </is>
       </c>
       <c r="K37" s="2" t="n">
-        <v>-8.047599999999999</v>
+        <v>-9.6204</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>-34.877</v>
+        <v>-42.0939</v>
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Recife</t>
+          <t>Remanso</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
@@ -7930,7 +7930,7 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>Viçosa do Ceará (CE)/ Piracuruca (PI)</t>
+          <t>Viçosa do Ceará</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
@@ -8225,10 +8225,10 @@
         </is>
       </c>
       <c r="K52" s="2" t="n">
-        <v>-15.7942</v>
+        <v>-9.898899999999999</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>-47.8822</v>
+        <v>-39.1486</v>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
@@ -8237,7 +8237,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Canudos</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Trilha Caminhos da Ibiapaba: manter apenas o ponto no Piauí
- Remove o local Viçosa do Ceará (CE); fica somente Piracuruca (PI)
- Vira ponto único: lat/lon, município e UF passam a Piracuruca/PI
  (estado "PI, CE" -> "PI"), sem array de locais
- ALT_LOCAIS com um só local agora também ajusta a UF; novo
  ENDERECO_OVERRIDES alinha o endereço ao Piauí
- Regenera iniciativas.js e a planilha-base limpa

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012qKixxvEYzG5RpjsaQG5UL
</commit_message>
<xml_diff>
--- a/PTE2026_base_limpa.xlsx
+++ b/PTE2026_base_limpa.xlsx
@@ -7914,14 +7914,14 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Rodovia Prefeito Vicente Miranda Filho, Viçosa do Ceará, Ceará, 62300-000</t>
+          <t>Parque Nacional de Sete Cidades, Piracuruca, PI, 64240-000</t>
         </is>
       </c>
       <c r="K50" s="2" t="n">
-        <v>-3.5619</v>
+        <v>-3.9285</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>-41.0922</v>
+        <v>-41.709</v>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
@@ -7930,12 +7930,12 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>Viçosa do Ceará</t>
+          <t>Piracuruca</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>PI, CE</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">

</xml_diff>